<commit_message>
Corregir bandas de markup en el Excel para que coincidan con la app real
PARAMETROS tenía los límites de banda mal (30k/60k/90k, redondeo a $50)
— no coinciden con la fórmula real que ya usa fmtPrecio() en
public/index.html (14k/18k/30k, redondeo a $500). Se corrigen los 4
valores (Tier1Limite, Tier2Limite, Tier3Limite, RedondeoA); los
multiplicadores 1.70/1.60/1.50/1.25 ya estaban bien. Todo lo demás del
archivo (fórmulas, nombres definidos, formato condicional, validación
de datos, freeze panes) queda intacto — se tocaron solo esas 4 celdas.
</commit_message>
<xml_diff>
--- a/interno/125cc_costeo_operativo.xlsx
+++ b/interno/125cc_costeo_operativo.xlsx
@@ -736,9 +736,6 @@
           <t>PARÁMETROS — 125cc Wine Bar (todo lo demás referencia esta hoja)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -768,9 +765,6 @@
           <t>OPERACIÓN</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -919,9 +913,6 @@
           <t>CARTA Y COSTO DE VINO</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -989,9 +980,6 @@
           <t>MARKUP ESCALONADO (precio de venta por copa)</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1000,7 +988,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>30000</v>
+        <v>14000</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
@@ -1032,7 +1020,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>60000</v>
+        <v>18000</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
@@ -1064,7 +1052,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>90000</v>
+        <v>30000</v>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
@@ -1112,7 +1100,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>50</v>
+        <v>500</v>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
@@ -1131,9 +1119,6 @@
           <t>MERMA — copas perdidas por botella (rendimiento real)</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1209,9 +1194,6 @@
           <t>COSTOS FIJOS MENSUALES (desglose editable)</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -1407,9 +1389,6 @@
           <t>COSTOS VARIABLES</t>
         </is>
       </c>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -1485,9 +1464,6 @@
           <t>OTROS INGRESOS</t>
         </is>
       </c>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -1587,9 +1563,6 @@
           <t>INFLACIÓN</t>
         </is>
       </c>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -1617,9 +1590,6 @@
           <t>ESTACIONALIDAD MAR DEL PLATA (índice s/mes base)</t>
         </is>
       </c>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -1790,19 +1760,6 @@
           <t>CARTA SEMANAL — 14 vinos simultáneos (renovación semanal)</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -2745,8 +2702,6 @@
           <t>TOTAL / PROMEDIO</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n"/>
-      <c r="C17" s="23" t="n"/>
       <c r="D17" s="24">
         <f>AVERAGE(D3:D16)</f>
         <v/>
@@ -2895,8 +2850,6 @@
           <t>MERMA Y CONTROL — rendimiento real de la botella</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -2904,8 +2857,6 @@
           <t>RENDIMIENTO REAL POR BOTELLA (copas efectivamente vendibles)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -3013,16 +2964,6 @@
           <t>IMPACTO EN EL MARGEN POR VINO (teórico 6 copas vs. rendimiento real)</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
-      <c r="K15" s="2" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3740,7 +3681,6 @@
           <t>PROMEDIO</t>
         </is>
       </c>
-      <c r="B31" s="25" t="n"/>
       <c r="C31" s="24">
         <f>AVERAGE(C17:C30)</f>
         <v/>
@@ -3840,13 +3780,6 @@
           <t>TAPEO — costeo por SKU</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -4306,13 +4239,6 @@
           <t>APORTE DEL TAPEO AL TICKET PROMEDIO</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -4421,9 +4347,6 @@
           <t>COSTOS FIJOS Y VARIABLES — desglose mensual</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -4431,9 +4354,6 @@
           <t>SUPUESTOS DE FACTURACIÓN BASE (para calcular variables)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -4485,9 +4405,6 @@
           <t>COSTOS FIJOS</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -4708,9 +4625,6 @@
           <t>COSTOS VARIABLES</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -4839,9 +4753,6 @@
           <t>PUNTO DE EQUILIBRIO — copas, pesos y personas por noche</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
@@ -4849,9 +4760,6 @@
           <t>SUPUESTOS COMUNES</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -5028,9 +4936,6 @@
           <t>EQUILIBRIO CON 5 NOCHES / SEMANA (costos fijos actuales)</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -5133,9 +5038,6 @@
           <t>EQUILIBRIO SIN 5ta NOCHE (referencia, 4 noches/semana)</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -5219,9 +5121,6 @@
           <t>EFECTO NETO DE LA 5ta NOCHE (mix 50% socias)</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="41" t="inlineStr">
@@ -5263,8 +5162,8 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A32:D32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5305,22 +5204,6 @@
           <t>RENTABILIDAD POR NOCHE — martes a sábado</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
-      <c r="N1" s="2" t="n"/>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="2" t="n"/>
-      <c r="Q1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -5956,18 +5839,6 @@
           <t>P&amp;L MENSUAL PROYECTADO — 12 meses, con estacionalidad de Mar del Plata</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-      <c r="M1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -6207,18 +6078,6 @@
           <t>INGRESOS</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -6501,18 +6360,6 @@
           <t>COSTOS</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -6905,18 +6752,6 @@
           <t>RESULTADO</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
@@ -7154,9 +6989,6 @@
           <t>ESCENARIOS — pesimista / base / optimista</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -7256,9 +7088,6 @@
           <t>PROYECCIÓN MENSUAL RESULTANTE</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">

</xml_diff>